<commit_message>
update: 2026/06/25 周四 10:56:21.45
</commit_message>
<xml_diff>
--- a/source/中心名单-2026-05.xlsx
+++ b/source/中心名单-2026-05.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="81">
   <si>
     <t>中心名称</t>
   </si>
@@ -267,6 +267,9 @@
   </si>
   <si>
     <t>滇西</t>
+  </si>
+  <si>
+    <t>湛江</t>
   </si>
 </sst>
 </file>
@@ -1272,7 +1275,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B77"/>
+  <dimension ref="A1:B78"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="16.8333333333333" customWidth="1"/>
@@ -1895,11 +1898,19 @@
         <v>63</v>
       </c>
     </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B57 B58 A59:B60" numberStoredAsText="1"/>
+    <ignoredError sqref="A59:B60 B58 A1:B57" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>